<commit_message>
doc: add enemey types and stats
</commit_message>
<xml_diff>
--- a/Assets/Docs/GameStats.xlsx
+++ b/Assets/Docs/GameStats.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="54">
   <si>
     <t xml:space="preserve">Object</t>
   </si>
@@ -50,12 +50,39 @@
     <t xml:space="preserve">BaseHP</t>
   </si>
   <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total Value inclusive fleet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tactic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Speed</t>
+  </si>
+  <si>
     <t xml:space="preserve">HP per Level</t>
   </si>
   <si>
+    <t xml:space="preserve">Fleet</t>
+  </si>
+  <si>
     <t xml:space="preserve">Weapons</t>
   </si>
   <si>
+    <t xml:space="preserve">Factory</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost Per Ship</t>
+  </si>
+  <si>
     <t xml:space="preserve">Damage</t>
   </si>
   <si>
@@ -68,13 +95,94 @@
     <t xml:space="preserve">Range</t>
   </si>
   <si>
+    <t xml:space="preserve">Produces</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time in s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Up To</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cannon Turret</t>
   </si>
   <si>
+    <t xml:space="preserve">Stay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
     <t xml:space="preserve">Small Cannon</t>
   </si>
   <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nearest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fast</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- </t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escort</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium Cannon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Player</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cruiser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missile Turret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battle Cruiser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrol  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large Cannon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Space Station</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battle Ship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Space Fortress</t>
   </si>
 </sst>
 </file>
@@ -84,7 +192,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,6 +223,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -130,12 +244,19 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="16">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -162,6 +283,34 @@
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin"/>
       <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
       <top/>
       <bottom style="thin"/>
       <diagonal/>
@@ -176,15 +325,8 @@
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right style="thin"/>
-      <top/>
+      <top style="thin"/>
       <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
-      <left style="thin"/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -195,9 +337,23 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right style="thin"/>
-      <top style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -227,7 +383,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -252,6 +408,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -260,39 +420,143 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -537,113 +801,1291 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:J5"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B2:U27"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="2" width="11.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="15.39"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="3.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="4.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="14.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="8.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="7.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="2" width="14.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="10.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="8.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="20.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="2" width="15.29"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="21" min="14" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="23" style="2" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
+      <c r="G2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="S2" s="8"/>
+      <c r="T2" s="8"/>
+      <c r="U2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="3"/>
       <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="6" t="s">
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="M3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="N3" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="P3" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q3" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="R3" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="S3" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="T3" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="U3" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J3" s="8" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="19" t="n">
+        <f aca="false">E4+J4*L4</f>
+        <v>11</v>
+      </c>
+      <c r="G4" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" s="21" t="str">
+        <f aca="false">C7</f>
+        <v>Escort</v>
+      </c>
+      <c r="L4" s="21" t="n">
+        <f aca="false">E7</f>
+        <v>3</v>
+      </c>
+      <c r="M4" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="N4" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q4" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="R4" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="S4" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="T4" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="U4" s="24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="17"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="N5" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q5" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="R5" s="25"/>
+      <c r="S5" s="26"/>
+      <c r="T5" s="26"/>
+      <c r="U5" s="27"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="L6" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="M6" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="N6" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="P6" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q6" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="R6" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="S6" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="T6" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="U6" s="34" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="29" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>40</v>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="J7" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="K7" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="M7" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="N7" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="P7" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q7" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="R7" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="S7" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="T7" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="U7" s="30" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>80</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <f aca="false">E8+J8*L8</f>
         <v>14</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="9" t="n">
+      <c r="G8" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="21" t="str">
+        <f aca="false">C7</f>
+        <v>Escort</v>
+      </c>
+      <c r="L8" s="21" t="n">
+        <f aca="false">E7</f>
+        <v>3</v>
+      </c>
+      <c r="M8" s="29" t="s">
+        <v>41</v>
+      </c>
+      <c r="N8" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="P8" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q8" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="R8" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="S8" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="T8" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="U8" s="34" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="17"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="N9" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="E4" s="10" t="n">
+      <c r="O9" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="P9" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q9" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="R9" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="S9" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="T9" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="U9" s="30" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="12" t="n">
+      <c r="C10" s="29" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="29" t="n">
+        <v>50</v>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="29" t="n">
+        <f aca="false">E10+J10*L10</f>
+        <v>17</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="I10" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="J10" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="28" t="str">
+        <f aca="false">C7</f>
+        <v>Escort</v>
+      </c>
+      <c r="L10" s="28" t="n">
+        <f aca="false">F7</f>
+        <v>3</v>
+      </c>
+      <c r="M10" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="N10" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="P10" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q10" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="R10" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="S10" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="T10" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="U10" s="30" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>125</v>
+      </c>
+      <c r="E11" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" s="36" t="n">
+        <f aca="false">J12*L12+J11*L11+E11</f>
+        <v>30</v>
+      </c>
+      <c r="G11" s="36" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="I11" s="20"/>
+      <c r="J11" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="37" t="str">
+        <f aca="false">C7</f>
+        <v>Escort</v>
+      </c>
+      <c r="L11" s="37" t="n">
+        <f aca="false">E7</f>
+        <v>3</v>
+      </c>
+      <c r="M11" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="N11" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="P11" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q11" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="R11" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="S11" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="T11" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="U11" s="38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="17"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="12"/>
-      <c r="I4" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="13" t="n">
+      <c r="K12" s="39" t="str">
+        <f aca="false">C8</f>
+        <v>Cruiser</v>
+      </c>
+      <c r="L12" s="39" t="n">
+        <f aca="false">E8</f>
+        <v>8</v>
+      </c>
+      <c r="M12" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="N12" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O12" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="P12" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q12" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="R12" s="35"/>
+      <c r="S12" s="36"/>
+      <c r="T12" s="36"/>
+      <c r="U12" s="38"/>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="17"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="41" t="s">
+        <v>35</v>
+      </c>
+      <c r="K13" s="41" t="s">
+        <v>35</v>
+      </c>
+      <c r="L13" s="41" t="s">
+        <v>35</v>
+      </c>
+      <c r="M13" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="N13" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="P13" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q13" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="R13" s="35"/>
+      <c r="S13" s="36"/>
+      <c r="T13" s="36"/>
+      <c r="U13" s="38"/>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="17"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="20"/>
+      <c r="J14" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="K14" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="L14" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="M14" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="N14" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="P14" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q14" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="R14" s="35"/>
+      <c r="S14" s="36"/>
+      <c r="T14" s="36"/>
+      <c r="U14" s="38"/>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="D15" s="36" t="n">
+        <v>300</v>
+      </c>
+      <c r="E15" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="F15" s="36" t="n">
+        <f aca="false">J15*L15+J16*L16+E15</f>
+        <v>74</v>
+      </c>
+      <c r="G15" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="36" t="s">
+        <v>29</v>
+      </c>
+      <c r="I15" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="J15" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="K15" s="37" t="str">
+        <f aca="false">C7</f>
+        <v>Escort</v>
+      </c>
+      <c r="L15" s="37" t="n">
+        <f aca="false">E7</f>
+        <v>3</v>
+      </c>
+      <c r="M15" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="N15" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="P15" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q15" s="24" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="9"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="15" t="n">
+      <c r="R15" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="S15" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="T15" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="U15" s="24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="36"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="39" t="str">
+        <f aca="false">C8</f>
+        <v>Cruiser</v>
+      </c>
+      <c r="L16" s="39" t="n">
+        <f aca="false">E8</f>
+        <v>8</v>
+      </c>
+      <c r="M16" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="N16" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="O16" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="P16" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q16" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="R16" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="S16" s="40" t="n">
+        <v>30</v>
+      </c>
+      <c r="T16" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="U16" s="34" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="36"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="36"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="41" t="s">
+        <v>35</v>
+      </c>
+      <c r="K17" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="L17" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="M17" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="N17" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="P17" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q17" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="R17" s="32"/>
+      <c r="S17" s="40"/>
+      <c r="T17" s="33"/>
+      <c r="U17" s="34"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="K18" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="L18" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="M18" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="N18" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O18" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="P18" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q18" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="R18" s="32"/>
+      <c r="S18" s="40"/>
+      <c r="T18" s="33"/>
+      <c r="U18" s="34"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="K19" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="L19" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="M19" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="N19" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" s="16" t="n">
+      <c r="O19" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="P19" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q19" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="R19" s="32"/>
+      <c r="S19" s="40"/>
+      <c r="T19" s="33"/>
+      <c r="U19" s="34"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="K20" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="L20" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="M20" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="N20" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O20" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="P20" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q20" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="R20" s="25"/>
+      <c r="S20" s="26"/>
+      <c r="T20" s="26"/>
+      <c r="U20" s="27"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" s="36" t="n">
+        <v>300</v>
+      </c>
+      <c r="E21" s="36" t="n">
+        <v>40</v>
+      </c>
+      <c r="F21" s="36" t="n">
+        <f aca="false">E21+J21*L21+J22*L22+L23*J23</f>
+        <v>106</v>
+      </c>
+      <c r="G21" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="H21" s="36" t="s">
+        <v>42</v>
+      </c>
+      <c r="I21" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="J21" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="K21" s="37" t="str">
+        <f aca="false">C7</f>
+        <v>Escort</v>
+      </c>
+      <c r="L21" s="37" t="n">
+        <f aca="false">E7</f>
+        <v>3</v>
+      </c>
+      <c r="M21" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="N21" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O21" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="P21" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q21" s="24" t="n">
         <v>6</v>
       </c>
+      <c r="R21" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="S21" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="T21" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="U21" s="24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="39" t="str">
+        <f aca="false">C8</f>
+        <v>Cruiser</v>
+      </c>
+      <c r="L22" s="39" t="n">
+        <f aca="false">E8</f>
+        <v>8</v>
+      </c>
+      <c r="M22" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="N22" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="O22" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="P22" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q22" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="R22" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="S22" s="40" t="n">
+        <v>30</v>
+      </c>
+      <c r="T22" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="U22" s="34" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="40" t="str">
+        <f aca="false">C11</f>
+        <v>Battle Cruiser</v>
+      </c>
+      <c r="L23" s="43" t="n">
+        <f aca="false">E11</f>
+        <v>10</v>
+      </c>
+      <c r="M23" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="N23" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O23" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="P23" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q23" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="R23" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="S23" s="40" t="n">
+        <v>30</v>
+      </c>
+      <c r="T23" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="U23" s="34" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="K24" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="L24" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="M24" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="N24" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O24" s="40" t="s">
+        <v>31</v>
+      </c>
+      <c r="P24" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q24" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="R24" s="32"/>
+      <c r="S24" s="40"/>
+      <c r="T24" s="40"/>
+      <c r="U24" s="34"/>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="K25" s="40" t="s">
+        <v>35</v>
+      </c>
+      <c r="L25" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="M25" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="N25" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="O25" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="P25" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q25" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="R25" s="32"/>
+      <c r="S25" s="40"/>
+      <c r="T25" s="40"/>
+      <c r="U25" s="34"/>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="36"/>
+      <c r="E26" s="36"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="K26" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="L26" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="M26" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="N26" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="P26" s="26" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q26" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="R26" s="25"/>
+      <c r="S26" s="26"/>
+      <c r="T26" s="26"/>
+      <c r="U26" s="27"/>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C27" s="2" t="s">
+        <v>53</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="61">
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
-    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:Q2"/>
+    <mergeCell ref="R2:T2"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="B11:B14"/>
+    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="D11:D14"/>
+    <mergeCell ref="E11:E14"/>
+    <mergeCell ref="F11:F14"/>
+    <mergeCell ref="G11:G14"/>
+    <mergeCell ref="H11:H14"/>
+    <mergeCell ref="I11:I14"/>
+    <mergeCell ref="R11:R14"/>
+    <mergeCell ref="S11:S14"/>
+    <mergeCell ref="T11:T14"/>
+    <mergeCell ref="U11:U14"/>
+    <mergeCell ref="B15:B20"/>
+    <mergeCell ref="C15:C20"/>
+    <mergeCell ref="D15:D20"/>
+    <mergeCell ref="E15:E20"/>
+    <mergeCell ref="F15:F20"/>
+    <mergeCell ref="G15:G20"/>
+    <mergeCell ref="H15:H20"/>
+    <mergeCell ref="I15:I20"/>
+    <mergeCell ref="B21:B26"/>
+    <mergeCell ref="C21:C26"/>
+    <mergeCell ref="D21:D26"/>
+    <mergeCell ref="E21:E26"/>
+    <mergeCell ref="F21:F26"/>
+    <mergeCell ref="G21:G26"/>
+    <mergeCell ref="H21:H26"/>
+    <mergeCell ref="I21:I26"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
feat: add particle effect to small enemy projectile
</commit_message>
<xml_diff>
--- a/Assets/Docs/GameStats.xlsx
+++ b/Assets/Docs/GameStats.xlsx
@@ -386,7 +386,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -396,10 +396,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -945,1731 +941,1729 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="8.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="20.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="2" width="15.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="21" min="14" style="2" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="22" min="22" style="3" width="11.53"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="23" style="2" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="14" style="2" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="I1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8" t="s">
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="9" t="s">
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="9"/>
-      <c r="T1" s="9"/>
-      <c r="U1" s="10"/>
+      <c r="S1" s="8"/>
+      <c r="T1" s="8"/>
+      <c r="U1" s="9"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="4"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="11" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="12" t="s">
+      <c r="K2" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="P2" s="14" t="s">
+      <c r="P2" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="Q2" s="12" t="s">
+      <c r="Q2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="R2" s="15" t="s">
+      <c r="R2" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="S2" s="16" t="s">
+      <c r="S2" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="T2" s="16" t="s">
+      <c r="T2" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="U2" s="17" t="s">
+      <c r="U2" s="16" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="18" t="n">
+      <c r="B3" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="20" t="n">
+      <c r="D3" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="21" t="n">
+      <c r="F3" s="20" t="n">
         <f aca="false">E3+J3*L3</f>
         <v>11</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="H3" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="J3" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="K3" s="23" t="str">
+      <c r="J3" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" s="22" t="str">
         <f aca="false">C6</f>
         <v>Escort</v>
       </c>
-      <c r="L3" s="23" t="n">
+      <c r="L3" s="22" t="n">
         <f aca="false">E6</f>
         <v>3</v>
       </c>
-      <c r="M3" s="24" t="s">
+      <c r="M3" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="N3" s="25" t="n">
+      <c r="N3" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="O3" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="25" t="s">
+      <c r="O3" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="Q3" s="26" t="n">
+      <c r="Q3" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="R3" s="24" t="s">
+      <c r="R3" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="S3" s="25" t="n">
+      <c r="S3" s="24" t="n">
         <v>30</v>
       </c>
-      <c r="T3" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="U3" s="26" t="s">
+      <c r="T3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="U3" s="25" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="18"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="27" t="s">
+      <c r="B4" s="17"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="N4" s="28" t="n">
+      <c r="N4" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="28" t="s">
+      <c r="O4" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="Q4" s="29" t="n">
+      <c r="Q4" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="R4" s="27"/>
-      <c r="S4" s="28"/>
-      <c r="T4" s="28"/>
-      <c r="U4" s="29"/>
+      <c r="R4" s="26"/>
+      <c r="S4" s="27"/>
+      <c r="T4" s="27"/>
+      <c r="U4" s="28"/>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="30" t="n">
+      <c r="B5" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="32" t="n">
+      <c r="D5" s="31" t="n">
         <v>20</v>
       </c>
-      <c r="E5" s="31" t="n">
+      <c r="E5" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="F5" s="32" t="n">
+      <c r="F5" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="31" t="s">
+      <c r="G5" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="32" t="s">
+      <c r="H5" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="33" t="n">
+      <c r="I5" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="J5" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="L5" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="M5" s="34" t="s">
+      <c r="J5" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="K5" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="L5" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="N5" s="31" t="n">
+      <c r="N5" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="O5" s="31" t="s">
-        <v>31</v>
-      </c>
-      <c r="P5" s="31" t="s">
+      <c r="O5" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="Q5" s="33" t="n">
+      <c r="Q5" s="32" t="n">
         <v>6</v>
       </c>
-      <c r="R5" s="35" t="s">
+      <c r="R5" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="S5" s="36" t="s">
+      <c r="S5" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="T5" s="36" t="s">
+      <c r="T5" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="U5" s="37" t="s">
+      <c r="U5" s="36" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" s="31" t="s">
+      <c r="B6" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="32" t="n">
+      <c r="D6" s="31" t="n">
         <v>40</v>
       </c>
-      <c r="E6" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="32" t="n">
-        <v>3</v>
-      </c>
-      <c r="G6" s="31" t="s">
+      <c r="E6" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="H6" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="I6" s="33" t="n">
+      <c r="H6" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="K6" s="30" t="s">
+      <c r="J6" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="K6" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="L6" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="M6" s="31" t="s">
+      <c r="L6" s="29" t="s">
+        <v>35</v>
+      </c>
+      <c r="M6" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="N6" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="O6" s="31" t="s">
+      <c r="N6" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="P6" s="31" t="s">
+      <c r="P6" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="Q6" s="33" t="n">
+      <c r="Q6" s="32" t="n">
         <v>7</v>
       </c>
-      <c r="R6" s="34" t="s">
+      <c r="R6" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="S6" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="T6" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="U6" s="33" t="s">
+      <c r="S6" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="T6" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="U6" s="32" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>80</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="38" t="n">
+      <c r="F7" s="37" t="n">
         <f aca="false">E7+J7*L7</f>
         <v>14</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="I7" s="22" t="n">
+      <c r="H7" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="I7" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="J7" s="23" t="n">
+      <c r="J7" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="K7" s="23" t="str">
+      <c r="K7" s="22" t="str">
         <f aca="false">C6</f>
         <v>Escort</v>
       </c>
-      <c r="L7" s="23" t="n">
+      <c r="L7" s="22" t="n">
         <f aca="false">E6</f>
         <v>3</v>
       </c>
-      <c r="M7" s="31" t="s">
+      <c r="M7" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="N7" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="O7" s="31" t="s">
+      <c r="N7" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="P7" s="31" t="s">
+      <c r="P7" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="Q7" s="33" t="n">
+      <c r="Q7" s="32" t="n">
         <v>7</v>
       </c>
-      <c r="R7" s="35" t="s">
+      <c r="R7" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="S7" s="36" t="s">
-        <v>35</v>
-      </c>
-      <c r="T7" s="36" t="s">
-        <v>35</v>
-      </c>
-      <c r="U7" s="37" t="s">
+      <c r="S7" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="T7" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="U7" s="36" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="18"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="19"/>
-      <c r="F8" s="38"/>
-      <c r="G8" s="19"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="34" t="s">
+      <c r="B8" s="17"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="N8" s="31" t="n">
+      <c r="N8" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="O8" s="31" t="s">
-        <v>31</v>
-      </c>
-      <c r="P8" s="31" t="s">
+      <c r="O8" s="30" t="s">
+        <v>31</v>
+      </c>
+      <c r="P8" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="Q8" s="33" t="n">
-        <v>3</v>
-      </c>
-      <c r="R8" s="34" t="s">
+      <c r="Q8" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="T8" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="U8" s="33" t="s">
+      <c r="S8" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="T8" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="U8" s="32" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="30" t="n">
+      <c r="B9" s="29" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="32" t="n">
+      <c r="D9" s="31" t="n">
         <v>50</v>
       </c>
-      <c r="E9" s="31" t="n">
+      <c r="E9" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="32" t="n">
+      <c r="F9" s="31" t="n">
         <f aca="false">E9+J9*L9</f>
         <v>17</v>
       </c>
-      <c r="G9" s="31" t="s">
+      <c r="G9" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="H9" s="32" t="s">
+      <c r="H9" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="I9" s="31" t="n">
+      <c r="I9" s="30" t="n">
         <v>10</v>
       </c>
-      <c r="J9" s="30" t="n">
+      <c r="J9" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="K9" s="30" t="str">
+      <c r="K9" s="29" t="str">
         <f aca="false">C6</f>
         <v>Escort</v>
       </c>
-      <c r="L9" s="30" t="n">
+      <c r="L9" s="29" t="n">
         <f aca="false">F6</f>
         <v>3</v>
       </c>
-      <c r="M9" s="31" t="s">
+      <c r="M9" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="N9" s="31" t="n">
+      <c r="N9" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="O9" s="31" t="s">
+      <c r="O9" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="P9" s="31" t="s">
+      <c r="P9" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="Q9" s="33" t="n">
+      <c r="Q9" s="32" t="n">
         <v>10</v>
       </c>
-      <c r="R9" s="34" t="s">
+      <c r="R9" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="S9" s="31" t="n">
+      <c r="S9" s="30" t="n">
         <v>20</v>
       </c>
-      <c r="T9" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="U9" s="33" t="s">
+      <c r="T9" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="U9" s="32" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="17" t="n">
         <v>125</v>
       </c>
-      <c r="E10" s="40" t="n">
+      <c r="E10" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="17" t="n">
         <f aca="false">J11*L11+J10*L10+E10</f>
         <v>30</v>
       </c>
-      <c r="G10" s="40" t="s">
+      <c r="G10" s="39" t="s">
         <v>48</v>
       </c>
-      <c r="H10" s="18" t="s">
+      <c r="H10" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="I10" s="22"/>
-      <c r="J10" s="41" t="n">
+      <c r="I10" s="21"/>
+      <c r="J10" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="K10" s="41" t="str">
+      <c r="K10" s="40" t="str">
         <f aca="false">C6</f>
         <v>Escort</v>
       </c>
-      <c r="L10" s="41" t="n">
+      <c r="L10" s="40" t="n">
         <f aca="false">E6</f>
         <v>3</v>
       </c>
-      <c r="M10" s="25" t="s">
+      <c r="M10" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="N10" s="25" t="n">
+      <c r="N10" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="O10" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="P10" s="25" t="s">
+      <c r="O10" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="Q10" s="26" t="n">
+      <c r="Q10" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="R10" s="39" t="s">
+      <c r="R10" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="S10" s="40" t="n">
+      <c r="S10" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="T10" s="40" t="n">
+      <c r="T10" s="39" t="n">
         <v>10</v>
       </c>
-      <c r="U10" s="42" t="s">
+      <c r="U10" s="41" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="18"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="43" t="n">
+      <c r="B11" s="17"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="39"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="K11" s="43" t="str">
+      <c r="K11" s="42" t="str">
         <f aca="false">C7</f>
         <v>Cruiser</v>
       </c>
-      <c r="L11" s="43" t="n">
+      <c r="L11" s="42" t="n">
         <f aca="false">E7</f>
         <v>8</v>
       </c>
-      <c r="M11" s="36" t="s">
+      <c r="M11" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="N11" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="O11" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="P11" s="36" t="s">
+      <c r="N11" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O11" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="P11" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q11" s="37" t="n">
+      <c r="Q11" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="R11" s="39"/>
-      <c r="S11" s="40"/>
-      <c r="T11" s="40"/>
-      <c r="U11" s="42"/>
+      <c r="R11" s="38"/>
+      <c r="S11" s="39"/>
+      <c r="T11" s="39"/>
+      <c r="U11" s="41"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="18"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="K12" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="L12" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="M12" s="36" t="s">
+      <c r="B12" s="17"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="39"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="K12" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="L12" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="M12" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="N12" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="O12" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="P12" s="36" t="s">
+      <c r="N12" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O12" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="P12" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q12" s="37" t="n">
+      <c r="Q12" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="R12" s="39"/>
-      <c r="S12" s="40"/>
-      <c r="T12" s="40"/>
-      <c r="U12" s="42"/>
+      <c r="R12" s="38"/>
+      <c r="S12" s="39"/>
+      <c r="T12" s="39"/>
+      <c r="U12" s="41"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="18"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="K13" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="L13" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="M13" s="28" t="s">
+      <c r="B13" s="17"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="K13" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="L13" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="M13" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="N13" s="28" t="n">
+      <c r="N13" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="O13" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="P13" s="28" t="s">
+      <c r="O13" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="P13" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="Q13" s="29" t="n">
+      <c r="Q13" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="R13" s="39"/>
-      <c r="S13" s="40"/>
-      <c r="T13" s="40"/>
-      <c r="U13" s="42"/>
+      <c r="R13" s="38"/>
+      <c r="S13" s="39"/>
+      <c r="T13" s="39"/>
+      <c r="U13" s="41"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="17" t="n">
         <v>300</v>
       </c>
-      <c r="E14" s="40" t="n">
+      <c r="E14" s="39" t="n">
         <v>20</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="17" t="n">
         <f aca="false">J14*L14+J15*L15+E14</f>
         <v>74</v>
       </c>
-      <c r="G14" s="40" t="s">
+      <c r="G14" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="18" t="s">
+      <c r="H14" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="I14" s="22" t="n">
+      <c r="I14" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="J14" s="41" t="n">
+      <c r="J14" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="K14" s="41" t="str">
+      <c r="K14" s="40" t="str">
         <f aca="false">C6</f>
         <v>Escort</v>
       </c>
-      <c r="L14" s="41" t="n">
+      <c r="L14" s="40" t="n">
         <f aca="false">E6</f>
         <v>3</v>
       </c>
-      <c r="M14" s="24" t="s">
+      <c r="M14" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="N14" s="25" t="n">
+      <c r="N14" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="O14" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="P14" s="25" t="s">
+      <c r="O14" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="P14" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="Q14" s="26" t="n">
+      <c r="Q14" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="R14" s="24" t="s">
+      <c r="R14" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="S14" s="25" t="n">
+      <c r="S14" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="T14" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="U14" s="26" t="s">
+      <c r="T14" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="U14" s="25" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="43" t="n">
-        <v>3</v>
-      </c>
-      <c r="K15" s="43" t="str">
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="39"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="39"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" s="42" t="str">
         <f aca="false">C7</f>
         <v>Cruiser</v>
       </c>
-      <c r="L15" s="43" t="n">
+      <c r="L15" s="42" t="n">
         <f aca="false">E7</f>
         <v>8</v>
       </c>
-      <c r="M15" s="35" t="s">
+      <c r="M15" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="N15" s="36" t="n">
+      <c r="N15" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="O15" s="36" t="s">
-        <v>31</v>
-      </c>
-      <c r="P15" s="36" t="s">
+      <c r="O15" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="P15" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q15" s="37" t="n">
+      <c r="Q15" s="36" t="n">
         <v>6</v>
       </c>
-      <c r="R15" s="35" t="s">
+      <c r="R15" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="S15" s="44" t="n">
+      <c r="S15" s="43" t="n">
         <v>30</v>
       </c>
-      <c r="T15" s="36" t="n">
+      <c r="T15" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="U15" s="37" t="s">
+      <c r="U15" s="36" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="K16" s="43" t="s">
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="39"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="42" t="s">
+        <v>35</v>
+      </c>
+      <c r="K16" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="L16" s="43" t="s">
+      <c r="L16" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="M16" s="35" t="s">
+      <c r="M16" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="N16" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="O16" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="P16" s="36" t="s">
+      <c r="N16" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="P16" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q16" s="37" t="n">
+      <c r="Q16" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="R16" s="35"/>
-      <c r="S16" s="44"/>
-      <c r="T16" s="36"/>
-      <c r="U16" s="37"/>
+      <c r="R16" s="34"/>
+      <c r="S16" s="43"/>
+      <c r="T16" s="35"/>
+      <c r="U16" s="36"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="43" t="s">
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="39"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="39"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="K17" s="43" t="s">
+      <c r="K17" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="L17" s="43" t="s">
+      <c r="L17" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="M17" s="35" t="s">
+      <c r="M17" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="N17" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="O17" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="P17" s="36" t="s">
+      <c r="N17" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="P17" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q17" s="37" t="n">
+      <c r="Q17" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="R17" s="35"/>
-      <c r="S17" s="44"/>
-      <c r="T17" s="36"/>
-      <c r="U17" s="37"/>
+      <c r="R17" s="34"/>
+      <c r="S17" s="43"/>
+      <c r="T17" s="35"/>
+      <c r="U17" s="36"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="43" t="s">
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="39"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="39"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="K18" s="43" t="s">
+      <c r="K18" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="L18" s="43" t="s">
+      <c r="L18" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="M18" s="35" t="s">
+      <c r="M18" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="N18" s="36" t="n">
+      <c r="N18" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="O18" s="36" t="s">
-        <v>31</v>
-      </c>
-      <c r="P18" s="36" t="s">
+      <c r="O18" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="P18" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="Q18" s="37" t="n">
+      <c r="Q18" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="R18" s="35"/>
-      <c r="S18" s="44"/>
-      <c r="T18" s="36"/>
-      <c r="U18" s="37"/>
+      <c r="R18" s="34"/>
+      <c r="S18" s="43"/>
+      <c r="T18" s="35"/>
+      <c r="U18" s="36"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="45" t="s">
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="K19" s="45" t="s">
+      <c r="K19" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="L19" s="45" t="s">
+      <c r="L19" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="M19" s="27" t="s">
+      <c r="M19" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="N19" s="28" t="n">
+      <c r="N19" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="O19" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="P19" s="28" t="s">
+      <c r="O19" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="P19" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="Q19" s="29" t="n">
+      <c r="Q19" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="R19" s="27"/>
-      <c r="S19" s="28"/>
-      <c r="T19" s="28"/>
-      <c r="U19" s="29"/>
+      <c r="R19" s="26"/>
+      <c r="S19" s="27"/>
+      <c r="T19" s="27"/>
+      <c r="U19" s="28"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="C20" s="39" t="s">
+      <c r="C20" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="17" t="n">
         <v>300</v>
       </c>
-      <c r="E20" s="40" t="n">
+      <c r="E20" s="39" t="n">
         <v>40</v>
       </c>
-      <c r="F20" s="18" t="n">
+      <c r="F20" s="17" t="n">
         <f aca="false">E20+J20*L20+J21*L21+L22*J22</f>
         <v>106</v>
       </c>
-      <c r="G20" s="40" t="s">
+      <c r="G20" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="H20" s="18" t="s">
+      <c r="H20" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="I20" s="22" t="n">
+      <c r="I20" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="J20" s="41" t="n">
+      <c r="J20" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="K20" s="41" t="str">
+      <c r="K20" s="40" t="str">
         <f aca="false">C6</f>
         <v>Escort</v>
       </c>
-      <c r="L20" s="41" t="n">
+      <c r="L20" s="40" t="n">
         <f aca="false">E6</f>
         <v>3</v>
       </c>
-      <c r="M20" s="24" t="s">
+      <c r="M20" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="N20" s="25" t="n">
+      <c r="N20" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="O20" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="P20" s="25" t="s">
+      <c r="O20" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="P20" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="Q20" s="26" t="n">
+      <c r="Q20" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="R20" s="24" t="s">
+      <c r="R20" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="S20" s="25" t="n">
+      <c r="S20" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="T20" s="25" t="n">
-        <v>3</v>
-      </c>
-      <c r="U20" s="26" t="s">
+      <c r="T20" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="U20" s="25" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="43" t="n">
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="39"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="39"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="K21" s="43" t="str">
+      <c r="K21" s="42" t="str">
         <f aca="false">C7</f>
         <v>Cruiser</v>
       </c>
-      <c r="L21" s="43" t="n">
+      <c r="L21" s="42" t="n">
         <f aca="false">E7</f>
         <v>8</v>
       </c>
-      <c r="M21" s="35" t="s">
+      <c r="M21" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="N21" s="36" t="n">
+      <c r="N21" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="O21" s="36" t="s">
-        <v>31</v>
-      </c>
-      <c r="P21" s="36" t="s">
+      <c r="O21" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="P21" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q21" s="37" t="n">
+      <c r="Q21" s="36" t="n">
         <v>6</v>
       </c>
-      <c r="R21" s="35" t="s">
+      <c r="R21" s="34" t="s">
         <v>39</v>
       </c>
-      <c r="S21" s="44" t="n">
+      <c r="S21" s="43" t="n">
         <v>30</v>
       </c>
-      <c r="T21" s="36" t="n">
+      <c r="T21" s="35" t="n">
         <v>5</v>
       </c>
-      <c r="U21" s="37" t="s">
+      <c r="U21" s="36" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="46" t="n">
+      <c r="B22" s="17"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="K22" s="44" t="str">
+      <c r="K22" s="43" t="str">
         <f aca="false">C10</f>
         <v>Battle Cruiser</v>
       </c>
-      <c r="L22" s="46" t="n">
+      <c r="L22" s="45" t="n">
         <f aca="false">E10</f>
         <v>10</v>
       </c>
-      <c r="M22" s="35" t="s">
+      <c r="M22" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="N22" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="O22" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="P22" s="36" t="s">
+      <c r="N22" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O22" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="P22" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q22" s="37" t="n">
+      <c r="Q22" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="R22" s="35" t="s">
+      <c r="R22" s="34" t="s">
         <v>44</v>
       </c>
-      <c r="S22" s="44" t="n">
+      <c r="S22" s="43" t="n">
         <v>30</v>
       </c>
-      <c r="T22" s="44" t="n">
+      <c r="T22" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="U22" s="37" t="s">
+      <c r="U22" s="36" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="K23" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="L23" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="M23" s="35" t="s">
+      <c r="B23" s="17"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="39"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="K23" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="L23" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="M23" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="N23" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="O23" s="44" t="s">
-        <v>31</v>
-      </c>
-      <c r="P23" s="36" t="s">
+      <c r="N23" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="O23" s="43" t="s">
+        <v>31</v>
+      </c>
+      <c r="P23" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="Q23" s="37" t="n">
+      <c r="Q23" s="36" t="n">
         <v>4</v>
       </c>
-      <c r="R23" s="35"/>
-      <c r="S23" s="44"/>
-      <c r="T23" s="44"/>
-      <c r="U23" s="37"/>
+      <c r="R23" s="34"/>
+      <c r="S23" s="43"/>
+      <c r="T23" s="43"/>
+      <c r="U23" s="36"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="40"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="K24" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="L24" s="46" t="s">
-        <v>35</v>
-      </c>
-      <c r="M24" s="35" t="s">
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="39"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="39"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="K24" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="L24" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="M24" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="N24" s="36" t="n">
+      <c r="N24" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="O24" s="36" t="s">
-        <v>31</v>
-      </c>
-      <c r="P24" s="36" t="s">
+      <c r="O24" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="P24" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="Q24" s="37" t="n">
+      <c r="Q24" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="R24" s="35"/>
-      <c r="S24" s="44"/>
-      <c r="T24" s="44"/>
-      <c r="U24" s="37"/>
+      <c r="R24" s="34"/>
+      <c r="S24" s="43"/>
+      <c r="T24" s="43"/>
+      <c r="U24" s="36"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="K25" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="L25" s="45" t="s">
-        <v>35</v>
-      </c>
-      <c r="M25" s="27" t="s">
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="39"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="39"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="K25" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="L25" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="M25" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="N25" s="28" t="n">
+      <c r="N25" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="O25" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="P25" s="28" t="s">
+      <c r="O25" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="P25" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="Q25" s="29" t="n">
+      <c r="Q25" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="R25" s="27"/>
-      <c r="S25" s="28"/>
-      <c r="T25" s="28"/>
-      <c r="U25" s="29"/>
+      <c r="R25" s="26"/>
+      <c r="S25" s="27"/>
+      <c r="T25" s="27"/>
+      <c r="U25" s="28"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="18" t="n">
+      <c r="B26" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="C26" s="39" t="s">
+      <c r="C26" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="18" t="n">
+      <c r="D26" s="17" t="n">
         <v>500</v>
       </c>
-      <c r="E26" s="40" t="n">
+      <c r="E26" s="39" t="n">
         <v>50</v>
       </c>
-      <c r="F26" s="18" t="n">
+      <c r="F26" s="17" t="n">
         <f aca="false">E26+J26*L26+J27*L27+J28*L28+J29*L29+J30*L30</f>
         <v>137</v>
       </c>
-      <c r="G26" s="40" t="s">
+      <c r="G26" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="H26" s="18" t="s">
+      <c r="H26" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="I26" s="22" t="n">
+      <c r="I26" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="J26" s="21" t="n">
+      <c r="J26" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="K26" s="47" t="str">
+      <c r="K26" s="46" t="str">
         <f aca="false">C6</f>
         <v>Escort</v>
       </c>
-      <c r="L26" s="21" t="n">
+      <c r="L26" s="20" t="n">
         <f aca="false">E6</f>
         <v>3</v>
       </c>
-      <c r="M26" s="48" t="s">
+      <c r="M26" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="N26" s="47" t="n">
+      <c r="N26" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="O26" s="47" t="s">
-        <v>31</v>
-      </c>
-      <c r="P26" s="47" t="s">
+      <c r="O26" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="P26" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="Q26" s="47" t="n">
+      <c r="Q26" s="46" t="n">
         <v>6</v>
       </c>
-      <c r="R26" s="49" t="s">
+      <c r="R26" s="48" t="s">
         <v>33</v>
       </c>
-      <c r="S26" s="47" t="n">
+      <c r="S26" s="46" t="n">
         <v>20</v>
       </c>
-      <c r="T26" s="47" t="n">
-        <v>3</v>
-      </c>
-      <c r="U26" s="42" t="s">
+      <c r="T26" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="U26" s="41" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="40"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="18"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="38" t="n">
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="K27" s="50" t="str">
+      <c r="K27" s="49" t="str">
         <f aca="false">C7</f>
         <v>Cruiser</v>
       </c>
-      <c r="L27" s="38" t="n">
+      <c r="L27" s="37" t="n">
         <f aca="false">E7</f>
         <v>8</v>
       </c>
-      <c r="M27" s="51" t="s">
+      <c r="M27" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="N27" s="51" t="n">
+      <c r="N27" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="O27" s="51" t="s">
-        <v>31</v>
-      </c>
-      <c r="P27" s="51" t="s">
+      <c r="O27" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="P27" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="Q27" s="51" t="n">
+      <c r="Q27" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="R27" s="52" t="s">
+      <c r="R27" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="S27" s="53" t="n">
+      <c r="S27" s="52" t="n">
         <v>30</v>
       </c>
-      <c r="T27" s="51" t="n">
+      <c r="T27" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="U27" s="54" t="s">
+      <c r="U27" s="53" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="22"/>
-      <c r="J28" s="38" t="n">
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="39"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="39"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="K28" s="50" t="str">
+      <c r="K28" s="49" t="str">
         <f aca="false">C10</f>
         <v>Battle Cruiser</v>
       </c>
-      <c r="L28" s="38" t="n">
+      <c r="L28" s="37" t="n">
         <f aca="false">E10</f>
         <v>10</v>
       </c>
-      <c r="M28" s="51" t="s">
+      <c r="M28" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="N28" s="55" t="n">
+      <c r="N28" s="54" t="n">
         <v>5</v>
       </c>
-      <c r="O28" s="55" t="s">
-        <v>31</v>
-      </c>
-      <c r="P28" s="55" t="s">
+      <c r="O28" s="54" t="s">
+        <v>31</v>
+      </c>
+      <c r="P28" s="54" t="s">
         <v>43</v>
       </c>
-      <c r="Q28" s="55" t="n">
+      <c r="Q28" s="54" t="n">
         <v>6</v>
       </c>
-      <c r="R28" s="52" t="s">
+      <c r="R28" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="S28" s="53" t="n">
+      <c r="S28" s="52" t="n">
         <v>30</v>
       </c>
-      <c r="T28" s="53" t="n">
+      <c r="T28" s="52" t="n">
         <v>2</v>
       </c>
-      <c r="U28" s="54" t="s">
+      <c r="U28" s="53" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="40"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="38" t="n">
-        <v>3</v>
-      </c>
-      <c r="K29" s="50" t="str">
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="39"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="39"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="K29" s="49" t="str">
         <f aca="false">C3</f>
         <v>Cannon Turret</v>
       </c>
-      <c r="L29" s="38" t="n">
+      <c r="L29" s="37" t="n">
         <f aca="false">E3</f>
         <v>2</v>
       </c>
-      <c r="M29" s="51" t="s">
+      <c r="M29" s="50" t="s">
         <v>49</v>
       </c>
-      <c r="N29" s="51" t="n">
+      <c r="N29" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="O29" s="51" t="s">
-        <v>31</v>
-      </c>
-      <c r="P29" s="51" t="s">
+      <c r="O29" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="P29" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="Q29" s="51" t="n">
+      <c r="Q29" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="R29" s="52" t="s">
+      <c r="R29" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="S29" s="50" t="n">
+      <c r="S29" s="49" t="n">
         <v>60</v>
       </c>
-      <c r="T29" s="50" t="n">
+      <c r="T29" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="U29" s="54" t="s">
+      <c r="U29" s="53" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="18"/>
-      <c r="E30" s="40"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="18"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="38" t="n">
-        <v>3</v>
-      </c>
-      <c r="K30" s="50" t="str">
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="39"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="21"/>
+      <c r="J30" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" s="49" t="str">
         <f aca="false">C9</f>
         <v>Missile Turret</v>
       </c>
-      <c r="L30" s="38" t="n">
+      <c r="L30" s="37" t="n">
         <f aca="false">E9</f>
         <v>5</v>
       </c>
-      <c r="M30" s="51" t="s">
+      <c r="M30" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="N30" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="O30" s="53" t="s">
-        <v>31</v>
-      </c>
-      <c r="P30" s="51" t="s">
+      <c r="N30" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="O30" s="52" t="s">
+        <v>31</v>
+      </c>
+      <c r="P30" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="Q30" s="51" t="n">
+      <c r="Q30" s="50" t="n">
         <v>4</v>
       </c>
-      <c r="R30" s="52"/>
-      <c r="S30" s="50"/>
-      <c r="T30" s="50"/>
-      <c r="U30" s="54"/>
+      <c r="R30" s="51"/>
+      <c r="S30" s="49"/>
+      <c r="T30" s="49"/>
+      <c r="U30" s="53"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="40"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="22"/>
-      <c r="J31" s="38" t="s">
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="39"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="K31" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="L31" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M31" s="51" t="s">
+      <c r="K31" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="L31" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="M31" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="N31" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="O31" s="53" t="s">
-        <v>31</v>
-      </c>
-      <c r="P31" s="51" t="s">
+      <c r="N31" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="O31" s="52" t="s">
+        <v>31</v>
+      </c>
+      <c r="P31" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="Q31" s="51" t="n">
+      <c r="Q31" s="50" t="n">
         <v>4</v>
       </c>
-      <c r="R31" s="52"/>
-      <c r="S31" s="50"/>
-      <c r="T31" s="50"/>
-      <c r="U31" s="54"/>
+      <c r="R31" s="51"/>
+      <c r="S31" s="49"/>
+      <c r="T31" s="49"/>
+      <c r="U31" s="53"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="18"/>
-      <c r="E32" s="40"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="40"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="22"/>
-      <c r="J32" s="38" t="s">
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="39"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="39"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="K32" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="L32" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M32" s="51" t="s">
+      <c r="K32" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="L32" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="M32" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="N32" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="O32" s="53" t="s">
-        <v>31</v>
-      </c>
-      <c r="P32" s="51" t="s">
+      <c r="N32" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="O32" s="52" t="s">
+        <v>31</v>
+      </c>
+      <c r="P32" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="Q32" s="51" t="n">
+      <c r="Q32" s="50" t="n">
         <v>4</v>
       </c>
-      <c r="R32" s="52"/>
-      <c r="S32" s="50"/>
-      <c r="T32" s="50"/>
-      <c r="U32" s="54"/>
+      <c r="R32" s="51"/>
+      <c r="S32" s="49"/>
+      <c r="T32" s="49"/>
+      <c r="U32" s="53"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="40"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="22"/>
-      <c r="J33" s="38" t="s">
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="39"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="K33" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="L33" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M33" s="51" t="s">
+      <c r="K33" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="L33" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="M33" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="N33" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="O33" s="53" t="s">
-        <v>31</v>
-      </c>
-      <c r="P33" s="51" t="s">
+      <c r="N33" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="O33" s="52" t="s">
+        <v>31</v>
+      </c>
+      <c r="P33" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="Q33" s="51" t="n">
+      <c r="Q33" s="50" t="n">
         <v>4</v>
       </c>
-      <c r="R33" s="52"/>
-      <c r="S33" s="50"/>
-      <c r="T33" s="50"/>
-      <c r="U33" s="54"/>
+      <c r="R33" s="51"/>
+      <c r="S33" s="49"/>
+      <c r="T33" s="49"/>
+      <c r="U33" s="53"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="18"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="40"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="38" t="s">
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="39"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="39"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="21"/>
+      <c r="J34" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="K34" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="L34" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M34" s="51" t="s">
+      <c r="K34" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="L34" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="M34" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="N34" s="51" t="n">
+      <c r="N34" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="O34" s="51" t="s">
-        <v>31</v>
-      </c>
-      <c r="P34" s="51" t="s">
+      <c r="O34" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="P34" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="Q34" s="51" t="n">
+      <c r="Q34" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="R34" s="52"/>
-      <c r="S34" s="50"/>
-      <c r="T34" s="50"/>
-      <c r="U34" s="54"/>
+      <c r="R34" s="51"/>
+      <c r="S34" s="49"/>
+      <c r="T34" s="49"/>
+      <c r="U34" s="53"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="18"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="40"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="40"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="22"/>
-      <c r="J35" s="38" t="s">
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="39"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="39"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="21"/>
+      <c r="J35" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="K35" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="L35" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M35" s="51" t="s">
+      <c r="K35" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="L35" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="M35" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="N35" s="55" t="n">
+      <c r="N35" s="54" t="n">
         <v>1</v>
       </c>
-      <c r="O35" s="55" t="s">
-        <v>31</v>
-      </c>
-      <c r="P35" s="55" t="s">
+      <c r="O35" s="54" t="s">
+        <v>31</v>
+      </c>
+      <c r="P35" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="Q35" s="55" t="n">
+      <c r="Q35" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="R35" s="52"/>
-      <c r="S35" s="50"/>
-      <c r="T35" s="50"/>
-      <c r="U35" s="54"/>
+      <c r="R35" s="51"/>
+      <c r="S35" s="49"/>
+      <c r="T35" s="49"/>
+      <c r="U35" s="53"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="18"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="40"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="40"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="38" t="s">
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="39"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="39"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="37" t="s">
         <v>38</v>
       </c>
-      <c r="K36" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="L36" s="38" t="s">
-        <v>35</v>
-      </c>
-      <c r="M36" s="51" t="s">
+      <c r="K36" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="L36" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="M36" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="N36" s="51" t="n">
+      <c r="N36" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="O36" s="51" t="s">
-        <v>31</v>
-      </c>
-      <c r="P36" s="51" t="s">
+      <c r="O36" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="P36" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="Q36" s="51" t="n">
+      <c r="Q36" s="50" t="n">
         <v>2</v>
       </c>
-      <c r="R36" s="52"/>
-      <c r="S36" s="50"/>
-      <c r="T36" s="50"/>
-      <c r="U36" s="54"/>
+      <c r="R36" s="51"/>
+      <c r="S36" s="49"/>
+      <c r="T36" s="49"/>
+      <c r="U36" s="53"/>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="18"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="40"/>
-      <c r="F37" s="18"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="18"/>
-      <c r="I37" s="22"/>
-      <c r="J37" s="56" t="s">
-        <v>35</v>
-      </c>
-      <c r="K37" s="57" t="s">
-        <v>35</v>
-      </c>
-      <c r="L37" s="56" t="s">
-        <v>35</v>
-      </c>
-      <c r="M37" s="57" t="s">
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="39"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="21"/>
+      <c r="J37" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="K37" s="56" t="s">
+        <v>35</v>
+      </c>
+      <c r="L37" s="55" t="s">
+        <v>35</v>
+      </c>
+      <c r="M37" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="N37" s="58" t="n">
+      <c r="N37" s="57" t="n">
         <v>1</v>
       </c>
-      <c r="O37" s="58" t="s">
-        <v>31</v>
-      </c>
-      <c r="P37" s="58" t="s">
+      <c r="O37" s="57" t="s">
+        <v>31</v>
+      </c>
+      <c r="P37" s="57" t="s">
         <v>32</v>
       </c>
-      <c r="Q37" s="58" t="n">
+      <c r="Q37" s="57" t="n">
         <v>2</v>
       </c>
-      <c r="R37" s="59"/>
-      <c r="S37" s="57"/>
-      <c r="T37" s="57"/>
-      <c r="U37" s="60"/>
+      <c r="R37" s="58"/>
+      <c r="S37" s="56"/>
+      <c r="T37" s="56"/>
+      <c r="U37" s="59"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="M38" s="36"/>
+      <c r="M38" s="35"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="M39" s="36"/>
+      <c r="M39" s="35"/>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>

</xml_diff>

<commit_message>
feat: add missile to ship
</commit_message>
<xml_diff>
--- a/Assets/Docs/GameStats.xlsx
+++ b/Assets/Docs/GameStats.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="SpriteOrder" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Enemies" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="PlayerWeapons" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="65">
   <si>
     <t xml:space="preserve">Object</t>
   </si>
@@ -186,6 +187,36 @@
   </si>
   <si>
     <t xml:space="preserve">BattleCruiser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main Cannon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defence Cannon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attack Drone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Armor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reload Speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.5</t>
   </si>
 </sst>
 </file>
@@ -386,7 +417,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="63">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -625,6 +656,18 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2746,4 +2789,158 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;KffffffSeite &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A3:F18"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="62" t="n">
+        <v>20</v>
+      </c>
+      <c r="C14" s="62" t="n">
+        <v>35</v>
+      </c>
+      <c r="D14" s="62" t="n">
+        <v>50</v>
+      </c>
+      <c r="E14" s="62" t="n">
+        <v>65</v>
+      </c>
+      <c r="F14" s="62" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="61" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="62" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="62" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="62" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="62" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="62" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="61" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="61" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="62" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="62" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="F17" s="62" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="62"/>
+      <c r="C18" s="62"/>
+      <c r="D18" s="62"/>
+      <c r="E18" s="62"/>
+      <c r="F18" s="62"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:F12"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Standard"&amp;12&amp;KffffffSeite &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
doc: add initial stats
</commit_message>
<xml_diff>
--- a/Assets/Docs/GameStats.xlsx
+++ b/Assets/Docs/GameStats.xlsx
@@ -10,7 +10,7 @@
   <sheets>
     <sheet name="SpriteOrder" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Enemies" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="PlayerWeapons" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="PlayerShipItems" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="71">
   <si>
     <t xml:space="preserve">Object</t>
   </si>
@@ -217,14 +217,33 @@
   </si>
   <si>
     <t xml:space="preserve">3.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recharge Delay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recharge per s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reduction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evade</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0.00\ %"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -417,7 +436,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -658,15 +677,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2796,21 +2819,24 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A3:F18"/>
+  <dimension ref="A3:F30"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.39"/>
+  </cols>
   <sheetData>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2925,15 +2951,241 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="62"/>
-      <c r="C18" s="62"/>
-      <c r="D18" s="62"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="62"/>
+      <c r="A18" s="60" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" s="60"/>
+      <c r="C18" s="60"/>
+      <c r="D18" s="60"/>
+      <c r="E18" s="60"/>
+      <c r="F18" s="60"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="61" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="62" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="62" t="n">
+        <v>25</v>
+      </c>
+      <c r="D20" s="62" t="n">
+        <v>40</v>
+      </c>
+      <c r="E20" s="62" t="n">
+        <v>55</v>
+      </c>
+      <c r="F20" s="62" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="B21" s="62" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" s="62" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="E21" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="62" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="61" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="60" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" s="60"/>
+      <c r="C23" s="60"/>
+      <c r="D23" s="60"/>
+      <c r="E23" s="60"/>
+      <c r="F23" s="60"/>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="61" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="62" t="n">
+        <v>50</v>
+      </c>
+      <c r="C25" s="62" t="n">
+        <v>60</v>
+      </c>
+      <c r="D25" s="62" t="n">
+        <v>70</v>
+      </c>
+      <c r="E25" s="62" t="n">
+        <v>80</v>
+      </c>
+      <c r="F25" s="62" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="61" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="62" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="60" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="60"/>
+      <c r="C27" s="60"/>
+      <c r="D27" s="60"/>
+      <c r="E27" s="60"/>
+      <c r="F27" s="60"/>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="62" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="61" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" s="62" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="62" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D29" s="62" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E29" s="62" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F29" s="62" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="61" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" s="62" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="63" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D30" s="63" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E30" s="63" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F30" s="63" t="n">
+        <v>0.2</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
     <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A27:F27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
feat: add missing stats for playership
</commit_message>
<xml_diff>
--- a/Assets/Docs/GameStats.xlsx
+++ b/Assets/Docs/GameStats.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="72">
   <si>
     <t xml:space="preserve">Object</t>
   </si>
@@ -192,25 +192,28 @@
     <t xml:space="preserve">Main Cannon</t>
   </si>
   <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reload Speed</t>
+  </si>
+  <si>
     <t xml:space="preserve">Defence Cannon</t>
   </si>
   <si>
     <t xml:space="preserve">Attack Drone</t>
   </si>
   <si>
-    <t xml:space="preserve">Level</t>
+    <t xml:space="preserve">Rebuild</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Armor</t>
   </si>
   <si>
     <t xml:space="preserve">5.5</t>
   </si>
   <si>
     <t xml:space="preserve">6.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Armor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reload Speed</t>
   </si>
   <si>
     <t xml:space="preserve">4.5</t>
@@ -245,7 +248,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00\ %"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -276,8 +279,16 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -287,13 +298,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFEEEEEE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDDDDD"/>
-        <bgColor rgb="FFCCFFCC"/>
+        <bgColor rgb="FFEEEEEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEEEEE"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -436,7 +453,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="73">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -677,19 +694,55 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="10" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -722,7 +775,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFEEEEEE"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -2819,373 +2872,663 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A3:F30"/>
+  <dimension ref="B3:G38"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="60" width="15.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15.39"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="3" style="60" width="11.53"/>
   </cols>
   <sheetData>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="61" t="s">
         <v>55</v>
       </c>
+      <c r="C3" s="61"/>
+      <c r="D3" s="61"/>
+      <c r="E3" s="61"/>
+      <c r="F3" s="61"/>
+      <c r="G3" s="61"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="64" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="62" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="E5" s="63" t="n">
+        <v>30</v>
+      </c>
+      <c r="F5" s="63" t="n">
+        <v>40</v>
+      </c>
+      <c r="G5" s="64" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="62" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="63" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="63" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" s="63" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" s="64" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="65" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="66" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E7" s="66" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F7" s="66" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G7" s="67" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="68" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="68"/>
+      <c r="F8" s="68"/>
+      <c r="G8" s="68"/>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="62" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="C9" s="63"/>
+      <c r="D9" s="63"/>
+      <c r="E9" s="63"/>
+      <c r="F9" s="63"/>
+      <c r="G9" s="64"/>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="62" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="63" t="n">
+        <v>15</v>
+      </c>
+      <c r="F10" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="G10" s="64" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="62" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="63" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="63" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G11" s="64" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="62" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="60" t="s">
+      <c r="C12" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="63" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E12" s="63" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F12" s="63" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G12" s="64" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="61" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="61"/>
+      <c r="D13" s="61"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="61"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="64" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="62" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="E15" s="63" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="G15" s="64" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="62" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="63" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E16" s="63" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F16" s="63" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G16" s="64" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="62" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="63" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D17" s="63" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E17" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="63" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G17" s="64" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="62" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="63" t="n">
+        <v>40</v>
+      </c>
+      <c r="D18" s="63" t="n">
+        <v>35</v>
+      </c>
+      <c r="E18" s="63" t="n">
+        <v>30</v>
+      </c>
+      <c r="F18" s="63" t="n">
+        <v>25</v>
+      </c>
+      <c r="G18" s="64" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="65" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" s="66" t="n">
+        <v>10</v>
+      </c>
+      <c r="E19" s="66" t="n">
+        <v>15</v>
+      </c>
+      <c r="F19" s="66" t="n">
+        <v>20</v>
+      </c>
+      <c r="G19" s="67" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="61" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="62" t="n">
+      <c r="C20" s="68"/>
+      <c r="D20" s="68"/>
+      <c r="E20" s="68"/>
+      <c r="F20" s="68"/>
+      <c r="G20" s="68"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="62" t="n">
+      <c r="D21" s="69" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="62" t="n">
+      <c r="E21" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F21" s="69" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="62" t="n">
+      <c r="G21" s="70" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="61" t="s">
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="62" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="62" t="n">
+      <c r="C22" s="69" t="n">
         <v>20</v>
       </c>
-      <c r="C14" s="62" t="n">
-        <v>35</v>
-      </c>
-      <c r="D14" s="62" t="n">
+      <c r="D22" s="69" t="n">
+        <v>35</v>
+      </c>
+      <c r="E22" s="69" t="n">
         <v>50</v>
       </c>
-      <c r="E14" s="62" t="n">
+      <c r="F22" s="69" t="n">
         <v>65</v>
       </c>
-      <c r="F14" s="62" t="n">
+      <c r="G22" s="70" t="n">
         <v>80</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="61" t="s">
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="62" t="n">
+      <c r="C23" s="69" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="62" t="s">
-        <v>59</v>
-      </c>
-      <c r="D15" s="62" t="n">
+      <c r="D23" s="69" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="69" t="n">
         <v>6</v>
       </c>
-      <c r="E15" s="62" t="s">
+      <c r="F23" s="69" t="s">
+        <v>63</v>
+      </c>
+      <c r="G23" s="70" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="62" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="70" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="62" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="69" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="69" t="s">
+        <v>65</v>
+      </c>
+      <c r="G25" s="70" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="61"/>
+      <c r="D26" s="61"/>
+      <c r="E26" s="61"/>
+      <c r="F26" s="61"/>
+      <c r="G26" s="61"/>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B27" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G27" s="70" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="D28" s="69" t="n">
+        <v>25</v>
+      </c>
+      <c r="E28" s="69" t="n">
+        <v>40</v>
+      </c>
+      <c r="F28" s="69" t="n">
+        <v>55</v>
+      </c>
+      <c r="G28" s="70" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="62" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="70" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="65" t="s">
+        <v>68</v>
+      </c>
+      <c r="C30" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E30" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="28" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="68" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="68"/>
+      <c r="D31" s="68"/>
+      <c r="E31" s="68"/>
+      <c r="F31" s="68"/>
+      <c r="G31" s="68"/>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C32" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" s="70" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" s="69" t="n">
+        <v>50</v>
+      </c>
+      <c r="D33" s="69" t="n">
         <v>60</v>
       </c>
-      <c r="F15" s="62" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="61" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" s="62" t="n">
+      <c r="E33" s="69" t="n">
+        <v>70</v>
+      </c>
+      <c r="F33" s="69" t="n">
+        <v>80</v>
+      </c>
+      <c r="G33" s="70" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="62" t="n">
+      <c r="E34" s="69" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="62" t="n">
+      <c r="F34" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="62" t="n">
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="61" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" s="61"/>
+      <c r="D35" s="61"/>
+      <c r="E35" s="61"/>
+      <c r="F35" s="61"/>
+      <c r="G35" s="61"/>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C36" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G36" s="70" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="61" t="s">
-        <v>62</v>
-      </c>
-      <c r="B17" s="62" t="n">
-        <v>5</v>
-      </c>
-      <c r="C17" s="62" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" s="62" t="n">
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="62" t="s">
+        <v>12</v>
+      </c>
+      <c r="C37" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" s="69" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E37" s="69" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F37" s="69" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="G37" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="E17" s="62" t="s">
-        <v>64</v>
-      </c>
-      <c r="F17" s="62" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="60" t="s">
-        <v>65</v>
-      </c>
-      <c r="B18" s="60"/>
-      <c r="C18" s="60"/>
-      <c r="D18" s="60"/>
-      <c r="E18" s="60"/>
-      <c r="F18" s="60"/>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="61" t="s">
-        <v>58</v>
-      </c>
-      <c r="B19" s="62" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="E19" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="F19" s="62" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="61" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" s="62" t="n">
-        <v>10</v>
-      </c>
-      <c r="C20" s="62" t="n">
-        <v>25</v>
-      </c>
-      <c r="D20" s="62" t="n">
-        <v>40</v>
-      </c>
-      <c r="E20" s="62" t="n">
-        <v>55</v>
-      </c>
-      <c r="F20" s="62" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="61" t="s">
-        <v>66</v>
-      </c>
-      <c r="B21" s="62" t="n">
-        <v>6</v>
-      </c>
-      <c r="C21" s="62" t="n">
-        <v>5</v>
-      </c>
-      <c r="D21" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" s="62" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="61" t="s">
-        <v>67</v>
-      </c>
-      <c r="B22" s="62" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="E22" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="F22" s="62" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="60" t="s">
-        <v>61</v>
-      </c>
-      <c r="B23" s="60"/>
-      <c r="C23" s="60"/>
-      <c r="D23" s="60"/>
-      <c r="E23" s="60"/>
-      <c r="F23" s="60"/>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="61" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="62" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="D24" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="E24" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="F24" s="62" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="61" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25" s="62" t="n">
-        <v>50</v>
-      </c>
-      <c r="C25" s="62" t="n">
-        <v>60</v>
-      </c>
-      <c r="D25" s="62" t="n">
-        <v>70</v>
-      </c>
-      <c r="E25" s="62" t="n">
-        <v>80</v>
-      </c>
-      <c r="F25" s="62" t="n">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="61" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="62" t="n">
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C38" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="62" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="62" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="60" t="s">
-        <v>69</v>
-      </c>
-      <c r="B27" s="60"/>
-      <c r="C27" s="60"/>
-      <c r="D27" s="60"/>
-      <c r="E27" s="60"/>
-      <c r="F27" s="60"/>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="61" t="s">
-        <v>58</v>
-      </c>
-      <c r="B28" s="62" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="D28" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="E28" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="F28" s="62" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="61" t="s">
-        <v>12</v>
-      </c>
-      <c r="B29" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="C29" s="62" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="D29" s="62" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E29" s="62" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="F29" s="62" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="61" t="s">
-        <v>70</v>
-      </c>
-      <c r="B30" s="62" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="63" t="n">
+      <c r="D38" s="71" t="n">
         <v>0.05</v>
       </c>
-      <c r="D30" s="63" t="n">
+      <c r="E38" s="71" t="n">
         <v>0.1</v>
       </c>
-      <c r="E30" s="63" t="n">
+      <c r="F38" s="71" t="n">
         <v>0.15</v>
       </c>
-      <c r="F30" s="63" t="n">
+      <c r="G38" s="72" t="n">
         <v>0.2</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A27:F27"/>
+  <mergeCells count="7">
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B35:G35"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
feat: add stats for main cannon
</commit_message>
<xml_diff>
--- a/Assets/Docs/GameStats.xlsx
+++ b/Assets/Docs/GameStats.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="72">
   <si>
     <t xml:space="preserve">Object</t>
   </si>
@@ -2872,7 +2872,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B3:G38"/>
+  <dimension ref="B3:G37"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="60" width="15.39"/>
@@ -2931,604 +2931,584 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="62" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="63" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" s="63" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" s="63" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" s="63" t="n">
-        <v>8</v>
-      </c>
-      <c r="G6" s="64" t="n">
-        <v>9</v>
+      <c r="B6" s="65" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="66" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="66" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E6" s="66" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F6" s="66" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G6" s="67" t="n">
+        <v>0.6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="65" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="66" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="66" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E7" s="66" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F7" s="66" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="G7" s="67" t="n">
-        <v>0.6</v>
-      </c>
+      <c r="B7" s="68" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="68"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="68"/>
+      <c r="F7" s="68"/>
+      <c r="G7" s="68"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="68" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="68"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="68"/>
+      <c r="B8" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="63"/>
+      <c r="D8" s="63"/>
+      <c r="E8" s="63"/>
+      <c r="F8" s="63"/>
+      <c r="G8" s="64"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="62" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="63"/>
-      <c r="D9" s="63"/>
-      <c r="E9" s="63"/>
-      <c r="F9" s="63"/>
-      <c r="G9" s="64"/>
+        <v>20</v>
+      </c>
+      <c r="C9" s="63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="63" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="63" t="n">
+        <v>15</v>
+      </c>
+      <c r="F9" s="63" t="n">
+        <v>20</v>
+      </c>
+      <c r="G9" s="64" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="62" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C10" s="63" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D10" s="63" t="n">
-        <v>10</v>
+        <v>1.5</v>
       </c>
       <c r="E10" s="63" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F10" s="63" t="n">
-        <v>20</v>
+        <v>2.5</v>
       </c>
       <c r="G10" s="64" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="62" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="C11" s="63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="63" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E11" s="63" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F11" s="63" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G11" s="64" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="61" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="63" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="E11" s="63" t="n">
+      <c r="D13" s="63" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="63" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G11" s="64" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="62" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="63" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="63" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="E12" s="63" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="F12" s="63" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G12" s="64" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="61" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" s="61"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="61"/>
-      <c r="F13" s="61"/>
-      <c r="G13" s="61"/>
+      <c r="E13" s="63" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="63" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="64" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="62" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="C14" s="63" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D14" s="63" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E14" s="63" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="F14" s="63" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="G14" s="64" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="62" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="C15" s="63" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D15" s="63" t="n">
-        <v>10</v>
+        <v>1.8</v>
       </c>
       <c r="E15" s="63" t="n">
-        <v>15</v>
+        <v>1.6</v>
       </c>
       <c r="F15" s="63" t="n">
-        <v>20</v>
+        <v>1.4</v>
       </c>
       <c r="G15" s="64" t="n">
-        <v>25</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="62" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="C16" s="63" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D16" s="63" t="n">
-        <v>1.8</v>
+        <v>0.75</v>
       </c>
       <c r="E16" s="63" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="F16" s="63" t="n">
-        <v>1.4</v>
+        <v>1.25</v>
       </c>
       <c r="G16" s="64" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="62" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="C17" s="63" t="n">
-        <v>0.5</v>
+        <v>40</v>
       </c>
       <c r="D17" s="63" t="n">
-        <v>0.75</v>
+        <v>35</v>
       </c>
       <c r="E17" s="63" t="n">
+        <v>30</v>
+      </c>
+      <c r="F17" s="63" t="n">
+        <v>25</v>
+      </c>
+      <c r="G17" s="64" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="65" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="66" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="66" t="n">
+        <v>10</v>
+      </c>
+      <c r="E18" s="66" t="n">
+        <v>15</v>
+      </c>
+      <c r="F18" s="66" t="n">
+        <v>20</v>
+      </c>
+      <c r="G18" s="67" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="68" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="68"/>
+      <c r="D19" s="68"/>
+      <c r="E19" s="68"/>
+      <c r="F19" s="68"/>
+      <c r="G19" s="68"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C20" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="63" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G17" s="64" t="n">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="62" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" s="63" t="n">
-        <v>40</v>
-      </c>
-      <c r="D18" s="63" t="n">
-        <v>35</v>
-      </c>
-      <c r="E18" s="63" t="n">
-        <v>30</v>
-      </c>
-      <c r="F18" s="63" t="n">
-        <v>25</v>
-      </c>
-      <c r="G18" s="64" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="65" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="66" t="n">
+      <c r="D20" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="70" t="n">
         <v>5</v>
       </c>
-      <c r="D19" s="66" t="n">
-        <v>10</v>
-      </c>
-      <c r="E19" s="66" t="n">
-        <v>15</v>
-      </c>
-      <c r="F19" s="66" t="n">
-        <v>20</v>
-      </c>
-      <c r="G19" s="67" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="68" t="s">
-        <v>46</v>
-      </c>
-      <c r="C20" s="68"/>
-      <c r="D20" s="68"/>
-      <c r="E20" s="68"/>
-      <c r="F20" s="68"/>
-      <c r="G20" s="68"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="62" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="C21" s="69" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D21" s="69" t="n">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="E21" s="69" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="F21" s="69" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="G21" s="70" t="n">
-        <v>5</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="62" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C22" s="69" t="n">
-        <v>20</v>
-      </c>
-      <c r="D22" s="69" t="n">
-        <v>35</v>
+        <v>5</v>
+      </c>
+      <c r="D22" s="69" t="s">
+        <v>62</v>
       </c>
       <c r="E22" s="69" t="n">
-        <v>50</v>
-      </c>
-      <c r="F22" s="69" t="n">
-        <v>65</v>
+        <v>6</v>
+      </c>
+      <c r="F22" s="69" t="s">
+        <v>63</v>
       </c>
       <c r="G22" s="70" t="n">
-        <v>80</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="62" t="s">
-        <v>23</v>
+        <v>61</v>
       </c>
       <c r="C23" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G23" s="70" t="n">
         <v>5</v>
-      </c>
-      <c r="D23" s="69" t="s">
-        <v>62</v>
-      </c>
-      <c r="E23" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="F23" s="69" t="s">
-        <v>63</v>
-      </c>
-      <c r="G23" s="70" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="62" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C24" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" s="69" t="s">
+        <v>64</v>
+      </c>
+      <c r="E24" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="F24" s="69" t="s">
+        <v>65</v>
+      </c>
+      <c r="G24" s="70" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="61" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" s="61"/>
+      <c r="D25" s="61"/>
+      <c r="E25" s="61"/>
+      <c r="F25" s="61"/>
+      <c r="G25" s="61"/>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="69" t="n">
+      <c r="D26" s="69" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="69" t="n">
-        <v>3</v>
-      </c>
-      <c r="F24" s="69" t="n">
+      <c r="E26" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="69" t="n">
         <v>4</v>
       </c>
-      <c r="G24" s="70" t="n">
+      <c r="G26" s="70" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="62" t="s">
-        <v>57</v>
-      </c>
-      <c r="C25" s="69" t="n">
-        <v>5</v>
-      </c>
-      <c r="D25" s="69" t="s">
-        <v>64</v>
-      </c>
-      <c r="E25" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="F25" s="69" t="s">
-        <v>65</v>
-      </c>
-      <c r="G25" s="70" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="61" t="s">
-        <v>66</v>
-      </c>
-      <c r="C26" s="61"/>
-      <c r="D26" s="61"/>
-      <c r="E26" s="61"/>
-      <c r="F26" s="61"/>
-      <c r="G26" s="61"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="62" t="s">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="C27" s="69" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D27" s="69" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E27" s="69" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="F27" s="69" t="n">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="G27" s="70" t="n">
-        <v>5</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="62" t="s">
-        <v>9</v>
+        <v>67</v>
       </c>
       <c r="C28" s="69" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D28" s="69" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="E28" s="69" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F28" s="69" t="n">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="G28" s="70" t="n">
-        <v>70</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="62" t="s">
-        <v>67</v>
-      </c>
-      <c r="C29" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="D29" s="69" t="n">
+      <c r="B29" s="65" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="E29" s="69" t="n">
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="68" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" s="68"/>
+      <c r="D30" s="68"/>
+      <c r="E30" s="68"/>
+      <c r="F30" s="68"/>
+      <c r="G30" s="68"/>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C31" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="69" t="n">
         <v>4</v>
       </c>
-      <c r="F29" s="69" t="n">
-        <v>3</v>
-      </c>
-      <c r="G29" s="70" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="65" t="s">
-        <v>68</v>
-      </c>
-      <c r="C30" s="27" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="F30" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="G30" s="28" t="n">
+      <c r="G31" s="70" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="68" t="s">
-        <v>61</v>
-      </c>
-      <c r="C31" s="68"/>
-      <c r="D31" s="68"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="68"/>
-      <c r="G31" s="68"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="62" t="s">
-        <v>56</v>
+        <v>9</v>
       </c>
       <c r="C32" s="69" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="D32" s="69" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="E32" s="69" t="n">
-        <v>3</v>
+        <v>70</v>
       </c>
       <c r="F32" s="69" t="n">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="G32" s="70" t="n">
-        <v>5</v>
+        <v>90</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="62" t="s">
-        <v>9</v>
+        <v>69</v>
       </c>
       <c r="C33" s="69" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D33" s="69" t="n">
-        <v>60</v>
+        <v>1</v>
       </c>
       <c r="E33" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="G33" s="70" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="61" t="s">
         <v>70</v>
       </c>
-      <c r="F33" s="69" t="n">
-        <v>80</v>
-      </c>
-      <c r="G33" s="70" t="n">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="62" t="s">
-        <v>69</v>
-      </c>
-      <c r="C34" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="69" t="n">
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="61"/>
+      <c r="F34" s="61"/>
+      <c r="G34" s="61"/>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C35" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="69" t="n">
+      <c r="D35" s="69" t="n">
         <v>2</v>
       </c>
-      <c r="F34" s="69" t="n">
-        <v>3</v>
-      </c>
-      <c r="G34" s="70" t="n">
+      <c r="E35" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" s="69" t="n">
         <v>4</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="61" t="s">
-        <v>70</v>
-      </c>
-      <c r="C35" s="61"/>
-      <c r="D35" s="61"/>
-      <c r="E35" s="61"/>
-      <c r="F35" s="61"/>
-      <c r="G35" s="61"/>
+      <c r="G35" s="70" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="62" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="C36" s="69" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D36" s="69" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="E36" s="69" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F36" s="69" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="G36" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="G36" s="70" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" s="69" t="n">
-        <v>3</v>
-      </c>
-      <c r="D37" s="69" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="E37" s="69" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F37" s="69" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="G37" s="70" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="65" t="s">
+      <c r="B37" s="65" t="s">
         <v>71</v>
       </c>
-      <c r="C38" s="27" t="n">
+      <c r="C37" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="D38" s="71" t="n">
+      <c r="D37" s="71" t="n">
         <v>0.05</v>
       </c>
-      <c r="E38" s="71" t="n">
+      <c r="E37" s="71" t="n">
         <v>0.1</v>
       </c>
-      <c r="F38" s="71" t="n">
+      <c r="F37" s="71" t="n">
         <v>0.15</v>
       </c>
-      <c r="G38" s="72" t="n">
+      <c r="G37" s="72" t="n">
         <v>0.2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="B31:G31"/>
-    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B34:G34"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
feat: add domain defence weapon
</commit_message>
<xml_diff>
--- a/Assets/Docs/GameStats.xlsx
+++ b/Assets/Docs/GameStats.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="71">
   <si>
     <t xml:space="preserve">Object</t>
   </si>
@@ -210,18 +210,6 @@
     <t xml:space="preserve">Armor</t>
   </si>
   <si>
-    <t xml:space="preserve">5.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.5</t>
-  </si>
-  <si>
     <t xml:space="preserve">Shield</t>
   </si>
   <si>
@@ -238,6 +226,15 @@
   </si>
   <si>
     <t xml:space="preserve">Evade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harvest Drone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harvest Speed</t>
   </si>
 </sst>
 </file>
@@ -2872,7 +2869,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B3:G37"/>
+  <dimension ref="B3:H42"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="60" width="15.39"/>
@@ -3217,14 +3214,14 @@
       <c r="C22" s="69" t="n">
         <v>5</v>
       </c>
-      <c r="D22" s="69" t="s">
-        <v>62</v>
+      <c r="D22" s="69" t="n">
+        <v>5.5</v>
       </c>
       <c r="E22" s="69" t="n">
         <v>6</v>
       </c>
-      <c r="F22" s="69" t="s">
-        <v>63</v>
+      <c r="F22" s="69" t="n">
+        <v>6.5</v>
       </c>
       <c r="G22" s="70" t="n">
         <v>7</v>
@@ -3257,14 +3254,14 @@
       <c r="C24" s="69" t="n">
         <v>5</v>
       </c>
-      <c r="D24" s="69" t="s">
-        <v>64</v>
+      <c r="D24" s="69" t="n">
+        <v>4.5</v>
       </c>
       <c r="E24" s="69" t="n">
         <v>4</v>
       </c>
-      <c r="F24" s="69" t="s">
-        <v>65</v>
+      <c r="F24" s="69" t="n">
+        <v>3.5</v>
       </c>
       <c r="G24" s="70" t="n">
         <v>3</v>
@@ -3272,7 +3269,7 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="61" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C25" s="61"/>
       <c r="D25" s="61"/>
@@ -3322,7 +3319,7 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="62" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C28" s="69" t="n">
         <v>6</v>
@@ -3342,7 +3339,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="65" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C29" s="27" t="n">
         <v>1</v>
@@ -3412,7 +3409,7 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="62" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C33" s="69" t="n">
         <v>0</v>
@@ -3432,7 +3429,7 @@
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="61" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C34" s="61"/>
       <c r="D34" s="61"/>
@@ -3482,7 +3479,7 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="65" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C37" s="27" t="n">
         <v>0</v>
@@ -3500,8 +3497,103 @@
         <v>0.2</v>
       </c>
     </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="61" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="61"/>
+      <c r="D38" s="61"/>
+      <c r="E38" s="61"/>
+      <c r="F38" s="61"/>
+      <c r="G38" s="61"/>
+      <c r="H38" s="0"/>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="62" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F39" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G39" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="H39" s="0"/>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B40" s="62" t="s">
+        <v>69</v>
+      </c>
+      <c r="C40" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="E40" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="G40" s="70" t="n">
+        <v>10</v>
+      </c>
+      <c r="H40" s="0"/>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B41" s="62" t="s">
+        <v>70</v>
+      </c>
+      <c r="C41" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G41" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="H41" s="0"/>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B42" s="65" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" s="27" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E42" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="27" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G42" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="H42" s="0"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="B12:G12"/>
@@ -3509,6 +3601,7 @@
     <mergeCell ref="B25:G25"/>
     <mergeCell ref="B30:G30"/>
     <mergeCell ref="B34:G34"/>
+    <mergeCell ref="B38:G38"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>